<commit_message>
fix(Hu_2020): recode interleaved blocks 4-8, restore ACC unified coding
- 42 600-row subjects re-validated as valid (Date timestamps monotonic;
  last 240 rows = 5 real interleaved matching blocks of 48 trials per paper)
- clean.R: recode Block 4-8 for rows 361-600 (48 rows per block, by time
  order); restore ACC unified coding (raw -1 no-response -> NA, 2 out-of-range
  -> -2, regression from 2026-09-01 clean.R extraction); guards for
  (Subject, Block, Trial) uniqueness
- Clean.csv regenerated: 44 subjects, 0 duplicate keys, ACC 0/1/NA/-2
- Dataset_inf.csv: numTrials 480->600, numBlocks 2->8, Note updated
  (byte-faithful, 3 cells only)
- Codebook Block/Trial descriptions + exp JSON detail updated
- validate_clean_csv.R: ACC_OK synced with unified coding (add -2/-3/-4)
</commit_message>
<xml_diff>
--- a/1_Data/Hu_2020_CollabraPsy/Codebook_Hu_2020_CollabraPsy_Exp1_Clean.xlsx
+++ b/1_Data/Hu_2020_CollabraPsy/Codebook_Hu_2020_CollabraPsy_Exp1_Clean.xlsx
@@ -468,12 +468,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Block number in the experiment; each block may contain practice or experimental trials</t>
+          <t>Block number in the matching task. Blocks 1-3 = formal blocks (120 trials each); Blocks 4-8 = five interleaved short matching blocks of 48 trials each (per paper 'five short interleaved perceptual-matching blocks of 48 trials'). Original program mis-coded blocks 4-8 as Block 1 (recoded 2026-09-02 by time order, 48 rows per block). Subjects 7302/7303 have blocks 1-3 only (no interleaved blocks).</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>1-8 (Number)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,12 +490,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Trial number within the block</t>
+          <t>Trial number within the block. Bin dimension merged into Trial (Trial = (Bin-1)*24 + Trial, recoded 2026-09-01/02): blocks 1-3 have Trials 1-120, blocks 4-8 have Trials 1-48.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>1-120 (blocks 1-3); 1-48 (blocks 4-8)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>